<commit_message>
Architecture: finalize Baseline v1.1 governed release
</commit_message>
<xml_diff>
--- a/architecture/released/v1.0/RELEASE-MANIFEST-v1.0.xlsx
+++ b/architecture/released/v1.0/RELEASE-MANIFEST-v1.0.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Manifest" sheetId="1" r:id="Rd01f31f084af49ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Manifest" sheetId="1" r:id="R0961f8bd702c4bed"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -141,17 +141,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ReleaseManifestv1_0" displayName="ReleaseManifestv1_0" ref="A5:H34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:H34"/>
-  <x:tableColumns count="8">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ReleaseManifestv1_0" displayName="ReleaseManifestv1_0" ref="A5:J55" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:J55"/>
+  <x:tableColumns count="10">
     <x:tableColumn id="1" name="Relative Path"/>
     <x:tableColumn id="2" name="Document Identifier"/>
     <x:tableColumn id="3" name="Document Title"/>
     <x:tableColumn id="4" name="Semantic Version"/>
     <x:tableColumn id="5" name="Status"/>
-    <x:tableColumn id="6" name="SHA-256 Checksum"/>
-    <x:tableColumn id="7" name="Superseded Document"/>
-    <x:tableColumn id="8" name="Approval Reference"/>
+    <x:tableColumn id="6" name="Current"/>
+    <x:tableColumn id="7" name="Authority"/>
+    <x:tableColumn id="8" name="SHA-256 Checksum"/>
+    <x:tableColumn id="9" name="Superseded Document"/>
+    <x:tableColumn id="10" name="Approval Reference"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -357,9 +359,11 @@
     <x:col min="3" max="3" width="48" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="68" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="35" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="38" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="68" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="35" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="38" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
@@ -373,6 +377,8 @@
       <x:c r="F1" s="3"/>
       <x:c r="G1" s="3"/>
       <x:c r="H1" s="3"/>
+      <x:c r="I1" s="3"/>
+      <x:c r="J1" s="3"/>
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="7" t="str">
@@ -385,6 +391,8 @@
       <x:c r="F2" s="7"/>
       <x:c r="G2" s="7"/>
       <x:c r="H2" s="7"/>
+      <x:c r="I2" s="7"/>
+      <x:c r="J2" s="7"/>
     </x:row>
     <x:row r="3" ht="23" customHeight="1">
       <x:c r="A3" s="10" t="str">
@@ -397,7 +405,7 @@
         <x:v>Artifact Count</x:v>
       </x:c>
       <x:c r="D3" s="10" t="n">
-        <x:v>29</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="E3" s="10" t="str">
         <x:v>Generated: 2026-08-08 | SHA-256 lowercase hexadecimal</x:v>
@@ -405,6 +413,8 @@
       <x:c r="F3" s="10"/>
       <x:c r="G3" s="10"/>
       <x:c r="H3" s="10"/>
+      <x:c r="I3" s="10"/>
+      <x:c r="J3" s="10"/>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
       <x:c r="A5" s="15" t="str">
@@ -423,12 +433,18 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="F5" s="15" t="str">
+        <x:v>Current</x:v>
+      </x:c>
+      <x:c r="G5" s="15" t="str">
+        <x:v>Authority</x:v>
+      </x:c>
+      <x:c r="H5" s="15" t="str">
         <x:v>SHA-256 Checksum</x:v>
       </x:c>
-      <x:c r="G5" s="15" t="str">
+      <x:c r="I5" s="15" t="str">
         <x:v>Superseded Document</x:v>
       </x:c>
-      <x:c r="H5" s="15" t="str">
+      <x:c r="J5" s="15" t="str">
         <x:v>Approval Reference</x:v>
       </x:c>
     </x:row>
@@ -448,181 +464,223 @@
       <x:c r="E6" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F6" s="20" t="str">
+      <x:c r="F6" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G6" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H6" s="20" t="str">
         <x:v>663cb6376f5b032928557ee9cfc0bca255e5dbfec89e7361931376bc1614e0da</x:v>
       </x:c>
-      <x:c r="G6" s="17" t="str">
+      <x:c r="I6" s="17" t="str">
         <x:v>Superseded by: AEM-001 v1.1</x:v>
       </x:c>
-      <x:c r="H6" s="17" t="str">
+      <x:c r="J6" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="32" customHeight="1">
       <x:c r="A7" s="17" t="str">
-        <x:v>architecture/released/v1.0/ASM-001_Assertion_Business_Capability_Specification_v1.0_FROZEN.docx</x:v>
+        <x:v>architecture/released/v1.0/ARCHITECTURE-CONSISTENCY-REPORT-v1.1_FROZEN.md</x:v>
       </x:c>
       <x:c r="B7" s="17" t="str">
-        <x:v>ASM-001</x:v>
+        <x:v>Architecture Consistency Report</x:v>
       </x:c>
       <x:c r="C7" s="17" t="str">
-        <x:v>ASM-001 Assertion Business Capability Specification</x:v>
+        <x:v>ARCHITECTURE-CONSISTENCY-REPORT-v1.1</x:v>
       </x:c>
       <x:c r="D7" s="19" t="str">
-        <x:v>1.0</x:v>
+        <x:v>1.1</x:v>
       </x:c>
       <x:c r="E7" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F7" s="20" t="str">
-        <x:v>70f02fb9d1b79b0a1a5757a6d2080544278a24f9d913df2940eb536243b95b52</x:v>
-      </x:c>
-      <x:c r="G7" s="17" t="str">
-        <x:v>Superseded by: ASM-001 v2.0</x:v>
-      </x:c>
-      <x:c r="H7" s="17" t="str">
+      <x:c r="F7" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G7" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H7" s="20" t="str">
+        <x:v>7701b242feb71937de8b7747aa55b7c8b44a52587d2fa427a0eaf9304cf71fcc</x:v>
+      </x:c>
+      <x:c r="I7" s="17" t="str">
+        <x:v>Superseded by: ACR-001 v1.2</x:v>
+      </x:c>
+      <x:c r="J7" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="32" customHeight="1">
       <x:c r="A8" s="17" t="str">
-        <x:v>architecture/released/v1.0/ASM-001_Assertion_Business_Capability_Specification_v2.0_FROZEN.docx</x:v>
+        <x:v>architecture/released/v1.0/ARCHITECTURE-DRIFT-REPORT-v1.1_FROZEN.md</x:v>
       </x:c>
       <x:c r="B8" s="17" t="str">
-        <x:v>ASM-001</x:v>
+        <x:v>Architecture Drift Report</x:v>
       </x:c>
       <x:c r="C8" s="17" t="str">
-        <x:v>ASM-001 Assertion Business Capability Specification</x:v>
+        <x:v>ARCHITECTURE-DRIFT-REPORT-v1.1</x:v>
       </x:c>
       <x:c r="D8" s="19" t="str">
-        <x:v>2.0</x:v>
+        <x:v>1.1</x:v>
       </x:c>
       <x:c r="E8" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F8" s="20" t="str">
-        <x:v>6720a69e73d59d56e0796159835ad00e53628478d5e706cfd1b8008dfb2a66ed</x:v>
-      </x:c>
-      <x:c r="G8" s="17" t="str">
-        <x:v>Superseded by: ASM-001 v2.1</x:v>
-      </x:c>
-      <x:c r="H8" s="17" t="str">
+      <x:c r="F8" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G8" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H8" s="20" t="str">
+        <x:v>7e5aaaab56631d0b9f3d9d203a76a726054b7a42fb5f2800858bc5c701217546</x:v>
+      </x:c>
+      <x:c r="I8" s="17" t="str">
+        <x:v>Superseded by: ADR-001 v1.2</x:v>
+      </x:c>
+      <x:c r="J8" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="32" customHeight="1">
       <x:c r="A9" s="17" t="str">
-        <x:v>architecture/released/v1.0/CDD_TEMPLATE_v2.0_FROZEN.docx</x:v>
+        <x:v>architecture/released/v1.0/ARCHITECTURE-GLOSSARY-v1.0_FROZEN.md</x:v>
       </x:c>
       <x:c r="B9" s="17" t="str">
-        <x:v>CDD Template</x:v>
+        <x:v>Architecture Glossary</x:v>
       </x:c>
       <x:c r="C9" s="17" t="str">
-        <x:v>CDD TEMPLATE</x:v>
+        <x:v>ARCHITECTURE-GLOSSARY-v1.0</x:v>
       </x:c>
       <x:c r="D9" s="19" t="str">
-        <x:v>2.0</x:v>
+        <x:v>1.0</x:v>
       </x:c>
       <x:c r="E9" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F9" s="20" t="str">
-        <x:v>25c1356a3610ddd369b66c01c3ed3cf65ef4b8abf06d7056cb6925c68d84b811</x:v>
-      </x:c>
-      <x:c r="G9" s="17" t="str">
-        <x:v>Superseded by: CDD Template v2.1</x:v>
-      </x:c>
-      <x:c r="H9" s="17" t="str">
+      <x:c r="F9" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G9" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H9" s="20" t="str">
+        <x:v>7da811d8832e98bf7d86346aed7b9c0a2aa0ee712118d70882f6d54c95ad719b</x:v>
+      </x:c>
+      <x:c r="I9" s="17" t="str">
+        <x:v>Superseded by: Architecture Glossary v1.1</x:v>
+      </x:c>
+      <x:c r="J9" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="32" customHeight="1">
       <x:c r="A10" s="17" t="str">
-        <x:v>architecture/released/v1.0/CDS-001_Codex_Development_Standard_v1.2_FROZEN.docx</x:v>
+        <x:v>architecture/released/v1.0/ASM-001_Assertion_Business_Capability_Specification_v1.0_FROZEN.docx</x:v>
       </x:c>
       <x:c r="B10" s="17" t="str">
-        <x:v>CDS-001</x:v>
+        <x:v>ASM-001</x:v>
       </x:c>
       <x:c r="C10" s="17" t="str">
-        <x:v>CDS-001 Codex Development Standard</x:v>
+        <x:v>ASM-001 Assertion Business Capability Specification</x:v>
       </x:c>
       <x:c r="D10" s="19" t="str">
-        <x:v>1.2</x:v>
+        <x:v>1.0</x:v>
       </x:c>
       <x:c r="E10" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F10" s="20" t="str">
-        <x:v>69360b0af61003c4326db9884d080c6a44adde8e5ea2551566c1802cd1a3ed23</x:v>
-      </x:c>
-      <x:c r="G10" s="17" t="str">
-        <x:v>Superseded by: CDS-001 v1.3</x:v>
-      </x:c>
-      <x:c r="H10" s="17" t="str">
+      <x:c r="F10" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G10" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H10" s="20" t="str">
+        <x:v>70f02fb9d1b79b0a1a5757a6d2080544278a24f9d913df2940eb536243b95b52</x:v>
+      </x:c>
+      <x:c r="I10" s="17" t="str">
+        <x:v>Superseded by: ASM-001 v2.0</x:v>
+      </x:c>
+      <x:c r="J10" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="32" customHeight="1">
       <x:c r="A11" s="17" t="str">
-        <x:v>architecture/released/v1.0/CDS-001-Authorized-Artifacts-Amendment.md</x:v>
+        <x:v>architecture/released/v1.0/ASM-001_Assertion_Business_Capability_Specification_v2.0_FROZEN.docx</x:v>
       </x:c>
       <x:c r="B11" s="17" t="str">
-        <x:v>CDS-001 Authorized Artifacts Amendment</x:v>
+        <x:v>ASM-001</x:v>
       </x:c>
       <x:c r="C11" s="17" t="str">
-        <x:v>CDS-001-Authorized-Artifacts-Amendment</x:v>
+        <x:v>ASM-001 Assertion Business Capability Specification</x:v>
       </x:c>
       <x:c r="D11" s="19" t="str">
-        <x:v>1.2</x:v>
+        <x:v>2.0</x:v>
       </x:c>
       <x:c r="E11" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F11" s="20" t="str">
-        <x:v>bf7844a5b6749b62c07850b979168225f566b909c15482f798718fde64aa583c</x:v>
-      </x:c>
-      <x:c r="G11" s="17" t="str">
-        <x:v>Superseded by: CDS-001 v1.3</x:v>
-      </x:c>
-      <x:c r="H11" s="17" t="str">
+      <x:c r="F11" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G11" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H11" s="20" t="str">
+        <x:v>6720a69e73d59d56e0796159835ad00e53628478d5e706cfd1b8008dfb2a66ed</x:v>
+      </x:c>
+      <x:c r="I11" s="17" t="str">
+        <x:v>Superseded by: ASM-001 v2.1</x:v>
+      </x:c>
+      <x:c r="J11" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="32" customHeight="1">
       <x:c r="A12" s="17" t="str">
-        <x:v>architecture/released/v1.0/DRM-001_Decision_Business_Capability_Specification_v1.0_FROZEN.docx</x:v>
+        <x:v>architecture/released/v1.0/ASM-001_Assertion_Business_Capability_Specification_v2.1_FROZEN.docx</x:v>
       </x:c>
       <x:c r="B12" s="17" t="str">
-        <x:v>DRM-001</x:v>
+        <x:v>ASM-001</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
-        <x:v>DRM-001 Decision Business Capability Specification</x:v>
+        <x:v>ASM-001 Assertion Business Capability Specification</x:v>
       </x:c>
       <x:c r="D12" s="19" t="str">
-        <x:v>1.0</x:v>
+        <x:v>2.1</x:v>
       </x:c>
       <x:c r="E12" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F12" s="20" t="str">
-        <x:v>3c5968a4d6fee4440eb1169fd281cc7c4773f31ca68464f6a49955c182f12055</x:v>
-      </x:c>
-      <x:c r="G12" s="17" t="str">
-        <x:v>Superseded by: DRM-001 v1.1</x:v>
-      </x:c>
-      <x:c r="H12" s="17" t="str">
+      <x:c r="F12" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G12" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H12" s="20" t="str">
+        <x:v>35171f4bb76502ddc8f32810550e9493e4d6be34a4d65e813a83588408fb9e92</x:v>
+      </x:c>
+      <x:c r="I12" s="17" t="str">
+        <x:v>Superseded by: ASM-001 v2.2</x:v>
+      </x:c>
+      <x:c r="J12" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="32" customHeight="1">
       <x:c r="A13" s="17" t="str">
-        <x:v>architecture/released/v1.0/EAH-001_ECOM_Architecture_Handbook_v1.1.docx</x:v>
+        <x:v>architecture/released/v1.0/BASELINE-RECORD-v1.1_FROZEN.md</x:v>
       </x:c>
       <x:c r="B13" s="17" t="str">
-        <x:v>EAH-001</x:v>
+        <x:v>Baseline Record</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
-        <x:v>EAH-001 ECOM Architecture Handbook</x:v>
+        <x:v>BASELINE-RECORD-v1.1</x:v>
       </x:c>
       <x:c r="D13" s="19" t="str">
         <x:v>1.1</x:v>
@@ -630,25 +688,31 @@
       <x:c r="E13" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F13" s="20" t="str">
-        <x:v>a420c61cae33a5891990d000fdabbf30b0b98de88e039d5d20a4b25d548e78ae</x:v>
-      </x:c>
-      <x:c r="G13" s="17" t="str">
-        <x:v>Superseded by: EAH-001 v1.2</x:v>
-      </x:c>
-      <x:c r="H13" s="17" t="str">
+      <x:c r="F13" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G13" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H13" s="20" t="str">
+        <x:v>f3a782fdc38b955c4a2c99b4283f2c9eafd64b2b546fa839fa56579adc299f7f</x:v>
+      </x:c>
+      <x:c r="I13" s="17" t="str">
+        <x:v>Superseded by: Baseline Record v1.2</x:v>
+      </x:c>
+      <x:c r="J13" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="32" customHeight="1">
       <x:c r="A14" s="17" t="str">
-        <x:v>architecture/released/v1.0/EAH-001_ECOM_Architecture_Handbook_v1.2_FROZEN.docx</x:v>
+        <x:v>architecture/released/v1.0/BASELINE-RECORD-v1.2_FROZEN.md</x:v>
       </x:c>
       <x:c r="B14" s="17" t="str">
-        <x:v>EAH-001</x:v>
+        <x:v>Baseline Record</x:v>
       </x:c>
       <x:c r="C14" s="17" t="str">
-        <x:v>EAH-001 ECOM Architecture Handbook</x:v>
+        <x:v>BASELINE-RECORD-v1.2</x:v>
       </x:c>
       <x:c r="D14" s="19" t="str">
         <x:v>1.2</x:v>
@@ -656,25 +720,31 @@
       <x:c r="E14" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F14" s="20" t="str">
-        <x:v>3b6a46616598e210cb43742f4d8789bbcba21ff089a204905cea9087ccf0a719</x:v>
-      </x:c>
-      <x:c r="G14" s="17" t="str">
-        <x:v>Superseded by: EAH-001 v1.3</x:v>
-      </x:c>
-      <x:c r="H14" s="17" t="str">
+      <x:c r="F14" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G14" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H14" s="20" t="str">
+        <x:v>254bf6ae74d972e6130c3f2ac868bfc7993b7d300bd7e849314e1a2f5e844169</x:v>
+      </x:c>
+      <x:c r="I14" s="17" t="str">
+        <x:v>Superseded by: Baseline Record v1.3</x:v>
+      </x:c>
+      <x:c r="J14" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="32" customHeight="1">
       <x:c r="A15" s="17" t="str">
-        <x:v>architecture/released/v1.0/EIC-001_Cognitive_Engine_Invocation_Architecture_v1.0_FROZEN.docx</x:v>
+        <x:v>architecture/released/v1.0/CAM-001_Canonical_Projection_Model_v1.0_FROZEN.docx</x:v>
       </x:c>
       <x:c r="B15" s="17" t="str">
-        <x:v>EIC-001</x:v>
+        <x:v>CAM-001</x:v>
       </x:c>
       <x:c r="C15" s="17" t="str">
-        <x:v>EIC-001 Cognitive Engine Invocation Architecture</x:v>
+        <x:v>CAM-001 Canonical Projection Model</x:v>
       </x:c>
       <x:c r="D15" s="19" t="str">
         <x:v>1.0</x:v>
@@ -682,51 +752,63 @@
       <x:c r="E15" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F15" s="20" t="str">
-        <x:v>bd3c128dc3bc4a5a616f7f186341dda3e64c641a8c7820eeea11be7d365f3c2c</x:v>
-      </x:c>
-      <x:c r="G15" s="17" t="str">
-        <x:v>Superseded by: EIC-001 v1.1</x:v>
-      </x:c>
-      <x:c r="H15" s="17" t="str">
+      <x:c r="F15" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G15" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H15" s="20" t="str">
+        <x:v>1ae6280a0b7ed79ba182b736c87ff55e9da225700dc2ded90b3a043f699f9c65</x:v>
+      </x:c>
+      <x:c r="I15" s="17" t="str">
+        <x:v>Superseded by: CAM-001 v1.1</x:v>
+      </x:c>
+      <x:c r="J15" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="32" customHeight="1">
       <x:c r="A16" s="17" t="str">
-        <x:v>architecture/released/v1.0/EOM-001_Cognitive_Engine_Orchestration_Architecture_v1.0_FROZEN.docx</x:v>
+        <x:v>architecture/released/v1.0/CDD_TEMPLATE_v2.0_FROZEN.docx</x:v>
       </x:c>
       <x:c r="B16" s="17" t="str">
-        <x:v>EOM-001</x:v>
+        <x:v>CDD Template</x:v>
       </x:c>
       <x:c r="C16" s="17" t="str">
-        <x:v>EOM-001 Cognitive Engine Orchestration Architecture</x:v>
+        <x:v>CDD TEMPLATE</x:v>
       </x:c>
       <x:c r="D16" s="19" t="str">
-        <x:v>1.0</x:v>
+        <x:v>2.0</x:v>
       </x:c>
       <x:c r="E16" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F16" s="20" t="str">
-        <x:v>ebcbb07cc90a5eec72e0751969b62c9ff12eeea19c17cf3a927d0b8043cdc877</x:v>
-      </x:c>
-      <x:c r="G16" s="17" t="str">
-        <x:v>Superseded by: EOM-001 v1.1</x:v>
-      </x:c>
-      <x:c r="H16" s="17" t="str">
+      <x:c r="F16" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G16" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H16" s="20" t="str">
+        <x:v>25c1356a3610ddd369b66c01c3ed3cf65ef4b8abf06d7056cb6925c68d84b811</x:v>
+      </x:c>
+      <x:c r="I16" s="17" t="str">
+        <x:v>Superseded by: CDD Template v2.1</x:v>
+      </x:c>
+      <x:c r="J16" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="32" customHeight="1">
       <x:c r="A17" s="17" t="str">
-        <x:v>architecture/released/v1.0/ERM-001_Enterprise_Entity_Resolution_Business_Capability_Specification_v2.1_FROZEN.docx</x:v>
+        <x:v>architecture/released/v1.0/CDD_TEMPLATE_v2.1_FROZEN.docx</x:v>
       </x:c>
       <x:c r="B17" s="17" t="str">
-        <x:v>ERM-001</x:v>
+        <x:v>CDD Template</x:v>
       </x:c>
       <x:c r="C17" s="17" t="str">
-        <x:v>ERM-001 Enterprise Entity Resolution Business Capability Specification</x:v>
+        <x:v>CDD TEMPLATE</x:v>
       </x:c>
       <x:c r="D17" s="19" t="str">
         <x:v>2.1</x:v>
@@ -734,25 +816,31 @@
       <x:c r="E17" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F17" s="20" t="str">
-        <x:v>836f25ebeb8ad081b54dae6954d6681a0aba0e4381173dded2794aae313c9698</x:v>
-      </x:c>
-      <x:c r="G17" s="17" t="str">
-        <x:v>Superseded by: ERM-001 v2.2</x:v>
-      </x:c>
-      <x:c r="H17" s="17" t="str">
+      <x:c r="F17" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G17" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H17" s="20" t="str">
+        <x:v>34bcaa1f37d166120e82ecff1a713057cd8c14bbf294f743e8c0cedb5a9e88e4</x:v>
+      </x:c>
+      <x:c r="I17" s="17" t="str">
+        <x:v>Superseded by: CDD Template v2.2 — non-compliant authorization model</x:v>
+      </x:c>
+      <x:c r="J17" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="32" customHeight="1">
       <x:c r="A18" s="17" t="str">
-        <x:v>architecture/released/v1.0/ESM-001_Cognitive_Engine_Execution_State_Architecture_v1.0_FROZEN.docx</x:v>
+        <x:v>architecture/released/v1.0/CDD-AUTHORIZATION-GAP-REVIEW-v1.0_FROZEN.md</x:v>
       </x:c>
       <x:c r="B18" s="17" t="str">
-        <x:v>ESM-001</x:v>
+        <x:v>CDD Authorization Gap Review</x:v>
       </x:c>
       <x:c r="C18" s="17" t="str">
-        <x:v>ESM-001 Cognitive Engine Execution State Architecture</x:v>
+        <x:v>CDD-AUTHORIZATION-GAP-REVIEW-v1.0</x:v>
       </x:c>
       <x:c r="D18" s="19" t="str">
         <x:v>1.0</x:v>
@@ -760,25 +848,31 @@
       <x:c r="E18" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F18" s="20" t="str">
-        <x:v>02fe31cbe62a4e130b9a81bc61763041d3e12f310bb66cc6b72b64646aa08c12</x:v>
-      </x:c>
-      <x:c r="G18" s="17" t="str">
-        <x:v>Superseded by: ESM-001 v1.1</x:v>
-      </x:c>
-      <x:c r="H18" s="17" t="str">
+      <x:c r="F18" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G18" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H18" s="20" t="str">
+        <x:v>2b4e29fcfc998768f98f8577f744d7e4c03c677c6c3a92f7783efe0314a9a844</x:v>
+      </x:c>
+      <x:c r="I18" s="17" t="str">
+        <x:v>Superseded by: CDD Authorization Gap Review v1.1</x:v>
+      </x:c>
+      <x:c r="J18" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="32" customHeight="1">
       <x:c r="A19" s="17" t="str">
-        <x:v>architecture/released/v1.0/KRM-001_Knowledge_Business_Capability_Specification_v1.2_FROZEN.docx</x:v>
+        <x:v>architecture/released/v1.0/CDS-001_Codex_Development_Standard_v1.2_FROZEN.docx</x:v>
       </x:c>
       <x:c r="B19" s="17" t="str">
-        <x:v>KRM-001</x:v>
+        <x:v>CDS-001</x:v>
       </x:c>
       <x:c r="C19" s="17" t="str">
-        <x:v>KRM-001 Knowledge Business Capability Specification</x:v>
+        <x:v>CDS-001 Codex Development Standard</x:v>
       </x:c>
       <x:c r="D19" s="19" t="str">
         <x:v>1.2</x:v>
@@ -786,179 +880,223 @@
       <x:c r="E19" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F19" s="20" t="str">
-        <x:v>411299c35ef7affd06dfa250eadddd60d1e5edbe9568933cfeb0ac0c7b8adde2</x:v>
-      </x:c>
-      <x:c r="G19" s="17" t="str">
-        <x:v>Superseded by: KRM-001 v1.3</x:v>
-      </x:c>
-      <x:c r="H19" s="17" t="str">
+      <x:c r="F19" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G19" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H19" s="20" t="str">
+        <x:v>69360b0af61003c4326db9884d080c6a44adde8e5ea2551566c1802cd1a3ed23</x:v>
+      </x:c>
+      <x:c r="I19" s="17" t="str">
+        <x:v>Superseded by: CDS-001 v1.3</x:v>
+      </x:c>
+      <x:c r="J19" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="32" customHeight="1">
       <x:c r="A20" s="17" t="str">
-        <x:v>architecture/released/v1.0/PAD-001_Product_Access_Architecture_v1.0_FROZEN.docx</x:v>
+        <x:v>architecture/released/v1.0/CDS-001-Authorized-Artifacts-Amendment.md</x:v>
       </x:c>
       <x:c r="B20" s="17" t="str">
-        <x:v>PAD-001 Product Access Architecture</x:v>
+        <x:v>CDS-001 Authorized Artifacts Amendment</x:v>
       </x:c>
       <x:c r="C20" s="17" t="str">
-        <x:v>PAD-001 Product Access Architecture</x:v>
+        <x:v>CDS-001-Authorized-Artifacts-Amendment</x:v>
       </x:c>
       <x:c r="D20" s="19" t="str">
-        <x:v>1.0</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="E20" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F20" s="20" t="str">
-        <x:v>705c30b0f4c8c755f3e6e46eba9c7974d0e827a664c573e23d05b13d9617a710</x:v>
-      </x:c>
-      <x:c r="G20" s="17" t="str">
-        <x:v>Superseded by: PAD-001 Protocol v1.1</x:v>
-      </x:c>
-      <x:c r="H20" s="17" t="str">
+      <x:c r="F20" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G20" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H20" s="20" t="str">
+        <x:v>bf7844a5b6749b62c07850b979168225f566b909c15482f798718fde64aa583c</x:v>
+      </x:c>
+      <x:c r="I20" s="17" t="str">
+        <x:v>Superseded by: CDS-001 v1.3 (consolidated)</x:v>
+      </x:c>
+      <x:c r="J20" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="32" customHeight="1">
       <x:c r="A21" s="17" t="str">
-        <x:v>architecture/released/v1.0/PAD-001_Product_Access_Protocol_Specification_v1.1_FROZEN.docx</x:v>
+        <x:v>architecture/released/v1.0/DRM-001_Decision_Business_Capability_Specification_v1.0_FROZEN.docx</x:v>
       </x:c>
       <x:c r="B21" s="17" t="str">
-        <x:v>PAD-001 Product Access Protocol</x:v>
+        <x:v>DRM-001</x:v>
       </x:c>
       <x:c r="C21" s="17" t="str">
-        <x:v>PAD-001 Product Access Protocol Specification</x:v>
+        <x:v>DRM-001 Decision Business Capability Specification</x:v>
       </x:c>
       <x:c r="D21" s="19" t="str">
-        <x:v>1.1</x:v>
+        <x:v>1.0</x:v>
       </x:c>
       <x:c r="E21" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F21" s="20" t="str">
-        <x:v>a19c88bfeaddc8d391bb46338f6f7c179d30af6154772082ebca4835b2ce5948</x:v>
-      </x:c>
-      <x:c r="G21" s="17" t="str">
-        <x:v>Superseded by: PAD-001 v1.2</x:v>
-      </x:c>
-      <x:c r="H21" s="17" t="str">
+      <x:c r="F21" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G21" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H21" s="20" t="str">
+        <x:v>3c5968a4d6fee4440eb1169fd281cc7c4773f31ca68464f6a49955c182f12055</x:v>
+      </x:c>
+      <x:c r="I21" s="17" t="str">
+        <x:v>Superseded by: DRM-001 v1.1</x:v>
+      </x:c>
+      <x:c r="J21" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="32" customHeight="1">
       <x:c r="A22" s="17" t="str">
-        <x:v>architecture/released/v1.0/PAD-001_Product_Access_Protocol_Specification_v1.2_FROZEN.docx</x:v>
+        <x:v>architecture/released/v1.0/DRM-001_Decision_Business_Capability_Specification_v1.1_FROZEN.docx</x:v>
       </x:c>
       <x:c r="B22" s="17" t="str">
-        <x:v>PAD-001 Product Access Protocol</x:v>
+        <x:v>DRM-001</x:v>
       </x:c>
       <x:c r="C22" s="17" t="str">
-        <x:v>PAD-001 Product Access Protocol Specification</x:v>
+        <x:v>DRM-001 Decision Business Capability Specification</x:v>
       </x:c>
       <x:c r="D22" s="19" t="str">
-        <x:v>1.2</x:v>
+        <x:v>1.1</x:v>
       </x:c>
       <x:c r="E22" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F22" s="20" t="str">
-        <x:v>496ee104092949a5245aca0a0a4862f3a14f7b244d6e3792c9b70ecf53172f2a</x:v>
-      </x:c>
-      <x:c r="G22" s="17" t="str">
-        <x:v>Superseded by: PAD-001 v1.3</x:v>
-      </x:c>
-      <x:c r="H22" s="17" t="str">
+      <x:c r="F22" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G22" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H22" s="20" t="str">
+        <x:v>20c0500dea5521f7fface35b3424aba4f1346460735b5217b38f5fc6713fb419</x:v>
+      </x:c>
+      <x:c r="I22" s="17" t="str">
+        <x:v>Superseded by: DRM-001 v1.2</x:v>
+      </x:c>
+      <x:c r="J22" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="32" customHeight="1">
       <x:c r="A23" s="17" t="str">
-        <x:v>architecture/released/v1.0/README.md</x:v>
+        <x:v>architecture/released/v1.0/EAH-001_ECOM_Architecture_Handbook_v1.1.docx</x:v>
       </x:c>
       <x:c r="B23" s="17" t="str">
-        <x:v>RELEASE-README</x:v>
+        <x:v>EAH-001</x:v>
       </x:c>
       <x:c r="C23" s="17" t="str">
-        <x:v>Architecture Release Baseline README</x:v>
+        <x:v>EAH-001 ECOM Architecture Handbook</x:v>
       </x:c>
       <x:c r="D23" s="19" t="str">
-        <x:v>v1.0</x:v>
+        <x:v>1.1</x:v>
       </x:c>
       <x:c r="E23" s="18" t="str">
-        <x:v>Historical</x:v>
-      </x:c>
-      <x:c r="F23" s="20" t="str">
-        <x:v>62dbb300a104238c4ec86ee58ff631a7359b6dca18b99ed6fe981685e194fdb8</x:v>
-      </x:c>
-      <x:c r="G23" s="17" t="str"/>
-      <x:c r="H23" s="17" t="str">
+        <x:v>Superseded</x:v>
+      </x:c>
+      <x:c r="F23" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G23" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H23" s="20" t="str">
+        <x:v>a420c61cae33a5891990d000fdabbf30b0b98de88e039d5d20a4b25d548e78ae</x:v>
+      </x:c>
+      <x:c r="I23" s="17" t="str">
+        <x:v>Superseded by: EAH-001 v1.2</x:v>
+      </x:c>
+      <x:c r="J23" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="32" customHeight="1">
       <x:c r="A24" s="17" t="str">
-        <x:v>architecture/released/v1.0/RFC-0001 - Enterprise Knowledge Specification v1.0.docx</x:v>
+        <x:v>architecture/released/v1.0/EAH-001_ECOM_Architecture_Handbook_v1.2_FROZEN.docx</x:v>
       </x:c>
       <x:c r="B24" s="17" t="str">
-        <x:v>RFC-0001</x:v>
+        <x:v>EAH-001</x:v>
       </x:c>
       <x:c r="C24" s="17" t="str">
-        <x:v>RFC-0001 - Enterprise Knowledge Specification</x:v>
+        <x:v>EAH-001 ECOM Architecture Handbook</x:v>
       </x:c>
       <x:c r="D24" s="19" t="str">
-        <x:v>1.0</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="E24" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F24" s="20" t="str">
-        <x:v>05be0b62e53744708d5268080406ec2e78c6ff5e541e657b3e11e3a98f18580c</x:v>
-      </x:c>
-      <x:c r="G24" s="17" t="str">
-        <x:v>Superseded by: RFC-012</x:v>
-      </x:c>
-      <x:c r="H24" s="17" t="str">
+      <x:c r="F24" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G24" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H24" s="20" t="str">
+        <x:v>3b6a46616598e210cb43742f4d8789bbcba21ff089a204905cea9087ccf0a719</x:v>
+      </x:c>
+      <x:c r="I24" s="17" t="str">
+        <x:v>Superseded by: EAH-001 v1.3</x:v>
+      </x:c>
+      <x:c r="J24" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="32" customHeight="1">
       <x:c r="A25" s="17" t="str">
-        <x:v>architecture/released/v1.0/RFC-0002 - Enterprise Ontology Specification v1.0.docx</x:v>
+        <x:v>architecture/released/v1.0/EAH-001_ECOM_Architecture_Handbook_v1.3_FROZEN.docx</x:v>
       </x:c>
       <x:c r="B25" s="17" t="str">
-        <x:v>RFC-0002</x:v>
+        <x:v>EAH-001</x:v>
       </x:c>
       <x:c r="C25" s="17" t="str">
-        <x:v>RFC-0002 - Enterprise Ontology Specification</x:v>
+        <x:v>EAH-001 ECOM Architecture Handbook</x:v>
       </x:c>
       <x:c r="D25" s="19" t="str">
-        <x:v>1.0</x:v>
+        <x:v>1.3</x:v>
       </x:c>
       <x:c r="E25" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F25" s="20" t="str">
-        <x:v>37c4efb92df9a5fd40d9b140971d6e482a06d712a6747ab455f3bc86b0e3aaff</x:v>
-      </x:c>
-      <x:c r="G25" s="17" t="str">
-        <x:v>Superseded by: RFC-012</x:v>
-      </x:c>
-      <x:c r="H25" s="17" t="str">
+      <x:c r="F25" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G25" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H25" s="20" t="str">
+        <x:v>2290ddd0850e6a4797db831112a9c39a838b7e00aecf5c7877d38935dea442fe</x:v>
+      </x:c>
+      <x:c r="I25" s="17" t="str">
+        <x:v>Superseded by: EAH-001 v1.4</x:v>
+      </x:c>
+      <x:c r="J25" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="32" customHeight="1">
       <x:c r="A26" s="17" t="str">
-        <x:v>architecture/released/v1.0/RFC-0003 - Institutional Acts Specification v1.0.docx</x:v>
+        <x:v>architecture/released/v1.0/EIC-001_Cognitive_Engine_Invocation_Architecture_v1.0_FROZEN.docx</x:v>
       </x:c>
       <x:c r="B26" s="17" t="str">
-        <x:v>RFC-0003</x:v>
+        <x:v>EIC-001</x:v>
       </x:c>
       <x:c r="C26" s="17" t="str">
-        <x:v>RFC-0003 - Institutional Acts Specification</x:v>
+        <x:v>EIC-001 Cognitive Engine Invocation Architecture</x:v>
       </x:c>
       <x:c r="D26" s="19" t="str">
         <x:v>1.0</x:v>
@@ -966,51 +1104,63 @@
       <x:c r="E26" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F26" s="20" t="str">
-        <x:v>2d130363c663e80c4ee4be3ad01961a69eed619d24bd5688f2cfa59017c72279</x:v>
-      </x:c>
-      <x:c r="G26" s="17" t="str">
-        <x:v>Superseded by: RFC-012</x:v>
-      </x:c>
-      <x:c r="H26" s="17" t="str">
+      <x:c r="F26" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G26" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H26" s="20" t="str">
+        <x:v>bd3c128dc3bc4a5a616f7f186341dda3e64c641a8c7820eeea11be7d365f3c2c</x:v>
+      </x:c>
+      <x:c r="I26" s="17" t="str">
+        <x:v>Superseded by: EIC-001 v1.1</x:v>
+      </x:c>
+      <x:c r="J26" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="32" customHeight="1">
       <x:c r="A27" s="17" t="str">
-        <x:v>architecture/released/v1.0/RFC-0004 - Enterprise Knowledge Graph Specification v1.0.docx</x:v>
+        <x:v>architecture/released/v1.0/EIC-001_Cognitive_Engine_Invocation_Architecture_v1.1_FROZEN.docx</x:v>
       </x:c>
       <x:c r="B27" s="17" t="str">
-        <x:v>RFC-0004</x:v>
+        <x:v>EIC-001</x:v>
       </x:c>
       <x:c r="C27" s="17" t="str">
-        <x:v>RFC-0004 - Enterprise Knowledge Graph Specification</x:v>
+        <x:v>EIC-001 Cognitive Engine Invocation Architecture</x:v>
       </x:c>
       <x:c r="D27" s="19" t="str">
-        <x:v>1.0</x:v>
+        <x:v>1.1</x:v>
       </x:c>
       <x:c r="E27" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F27" s="20" t="str">
-        <x:v>0f8162d2dceb1e1b544bb7bb2cd0eae11c6c07f84e2f3b81c30f6699927f0874</x:v>
-      </x:c>
-      <x:c r="G27" s="17" t="str">
-        <x:v>Superseded by: RFC-012</x:v>
-      </x:c>
-      <x:c r="H27" s="17" t="str">
+      <x:c r="F27" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G27" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H27" s="20" t="str">
+        <x:v>1c0c6d12ae6c495f00b41c2104ea629aadb535f7ce42b0262e48c265fb8c6abe</x:v>
+      </x:c>
+      <x:c r="I27" s="17" t="str">
+        <x:v>Superseded by: EIC-001 v1.2</x:v>
+      </x:c>
+      <x:c r="J27" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="32" customHeight="1">
       <x:c r="A28" s="17" t="str">
-        <x:v>architecture/released/v1.0/RFC-0005 - Decision Assembly Specification v1.0.docx</x:v>
+        <x:v>architecture/released/v1.0/EOM-001_Cognitive_Engine_Orchestration_Architecture_v1.0_FROZEN.docx</x:v>
       </x:c>
       <x:c r="B28" s="17" t="str">
-        <x:v>RFC-0005</x:v>
+        <x:v>EOM-001</x:v>
       </x:c>
       <x:c r="C28" s="17" t="str">
-        <x:v>RFC-0005 - Decision Assembly Specification</x:v>
+        <x:v>EOM-001 Cognitive Engine Orchestration Architecture</x:v>
       </x:c>
       <x:c r="D28" s="19" t="str">
         <x:v>1.0</x:v>
@@ -1018,77 +1168,95 @@
       <x:c r="E28" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F28" s="20" t="str">
-        <x:v>756eb0ee4d57cbd5795ca56f31ba3b479431eaf3e31abfd480e5d21765bbc8a5</x:v>
-      </x:c>
-      <x:c r="G28" s="17" t="str">
-        <x:v>Superseded by: RFC-012</x:v>
-      </x:c>
-      <x:c r="H28" s="17" t="str">
+      <x:c r="F28" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G28" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H28" s="20" t="str">
+        <x:v>ebcbb07cc90a5eec72e0751969b62c9ff12eeea19c17cf3a927d0b8043cdc877</x:v>
+      </x:c>
+      <x:c r="I28" s="17" t="str">
+        <x:v>Superseded by: EOM-001 v1.1</x:v>
+      </x:c>
+      <x:c r="J28" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="32" customHeight="1">
       <x:c r="A29" s="17" t="str">
-        <x:v>architecture/released/v1.0/RFC-0006 - Enterprise Memory Specification v1.0.docx</x:v>
+        <x:v>architecture/released/v1.0/EOM-001_Cognitive_Engine_Orchestration_Architecture_v1.1_FROZEN.docx</x:v>
       </x:c>
       <x:c r="B29" s="17" t="str">
-        <x:v>RFC-0006</x:v>
+        <x:v>EOM-001</x:v>
       </x:c>
       <x:c r="C29" s="17" t="str">
-        <x:v>RFC-0006 - Enterprise Memory Specification</x:v>
+        <x:v>EOM-001 Cognitive Engine Orchestration Architecture</x:v>
       </x:c>
       <x:c r="D29" s="19" t="str">
-        <x:v>1.0</x:v>
+        <x:v>1.1</x:v>
       </x:c>
       <x:c r="E29" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F29" s="20" t="str">
-        <x:v>853578f062a3f8d6662f50d6fa8535ce5c0c5e992ee14a7599432cfa3b6b6933</x:v>
-      </x:c>
-      <x:c r="G29" s="17" t="str">
-        <x:v>Superseded by: RFC-012</x:v>
-      </x:c>
-      <x:c r="H29" s="17" t="str">
+      <x:c r="F29" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G29" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H29" s="20" t="str">
+        <x:v>c23b29b90e83aab0d1c14404af818cc89acd9730ee2d496a04667cbbfdd6c87a</x:v>
+      </x:c>
+      <x:c r="I29" s="17" t="str">
+        <x:v>Superseded by: EOM-001 v1.2</x:v>
+      </x:c>
+      <x:c r="J29" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="32" customHeight="1">
       <x:c r="A30" s="17" t="str">
-        <x:v>architecture/released/v1.0/RFC-0007 - Enterprise Reasoning Specification v1.0.docx</x:v>
+        <x:v>architecture/released/v1.0/ERM-001_Enterprise_Entity_Resolution_Business_Capability_Specification_v2.1_FROZEN.docx</x:v>
       </x:c>
       <x:c r="B30" s="17" t="str">
-        <x:v>RFC-0007</x:v>
+        <x:v>ERM-001</x:v>
       </x:c>
       <x:c r="C30" s="17" t="str">
-        <x:v>RFC-0007 - Enterprise Reasoning Specification</x:v>
+        <x:v>ERM-001 Enterprise Entity Resolution Business Capability Specification</x:v>
       </x:c>
       <x:c r="D30" s="19" t="str">
-        <x:v>1.0</x:v>
+        <x:v>2.1</x:v>
       </x:c>
       <x:c r="E30" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F30" s="20" t="str">
-        <x:v>370b47e8fbfba8ec34afaf78e7cb4c11cd6b5ca19e8605f21a8649491e1712ed</x:v>
-      </x:c>
-      <x:c r="G30" s="17" t="str">
-        <x:v>Superseded by: RFC-012</x:v>
-      </x:c>
-      <x:c r="H30" s="17" t="str">
+      <x:c r="F30" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G30" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H30" s="20" t="str">
+        <x:v>836f25ebeb8ad081b54dae6954d6681a0aba0e4381173dded2794aae313c9698</x:v>
+      </x:c>
+      <x:c r="I30" s="17" t="str">
+        <x:v>Superseded by: ERM-001 v2.2</x:v>
+      </x:c>
+      <x:c r="J30" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="32" customHeight="1">
       <x:c r="A31" s="17" t="str">
-        <x:v>architecture/released/v1.0/RFC-0008 - Enterprise Decision Specification v1.0.docx</x:v>
+        <x:v>architecture/released/v1.0/ESM-001_Cognitive_Engine_Execution_State_Architecture_v1.0_FROZEN.docx</x:v>
       </x:c>
       <x:c r="B31" s="17" t="str">
-        <x:v>RFC-0008</x:v>
+        <x:v>ESM-001</x:v>
       </x:c>
       <x:c r="C31" s="17" t="str">
-        <x:v>RFC-0008 - Enterprise Decision Specification</x:v>
+        <x:v>ESM-001 Cognitive Engine Execution State Architecture</x:v>
       </x:c>
       <x:c r="D31" s="19" t="str">
         <x:v>1.0</x:v>
@@ -1096,51 +1264,63 @@
       <x:c r="E31" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F31" s="20" t="str">
-        <x:v>88850719c91374469a930ac5420232e45df78c821ad5515cb00dd7c6ebc45fcb</x:v>
-      </x:c>
-      <x:c r="G31" s="17" t="str">
-        <x:v>Superseded by: RFC-012</x:v>
-      </x:c>
-      <x:c r="H31" s="17" t="str">
+      <x:c r="F31" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G31" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H31" s="20" t="str">
+        <x:v>02fe31cbe62a4e130b9a81bc61763041d3e12f310bb66cc6b72b64646aa08c12</x:v>
+      </x:c>
+      <x:c r="I31" s="17" t="str">
+        <x:v>Superseded by: ESM-001 v1.1</x:v>
+      </x:c>
+      <x:c r="J31" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="32" customHeight="1">
       <x:c r="A32" s="17" t="str">
-        <x:v>architecture/released/v1.0/RFC-0009 - Enterprise Learning Specification v1.0.docx</x:v>
+        <x:v>architecture/released/v1.0/ESM-001_Cognitive_Engine_Execution_State_Architecture_v1.1_FROZEN.docx</x:v>
       </x:c>
       <x:c r="B32" s="17" t="str">
-        <x:v>RFC-0009</x:v>
+        <x:v>ESM-001</x:v>
       </x:c>
       <x:c r="C32" s="17" t="str">
-        <x:v>RFC-0009 - Enterprise Learning Specification</x:v>
+        <x:v>ESM-001 Cognitive Engine Execution State Architecture</x:v>
       </x:c>
       <x:c r="D32" s="19" t="str">
-        <x:v>1.0</x:v>
+        <x:v>1.1</x:v>
       </x:c>
       <x:c r="E32" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F32" s="20" t="str">
-        <x:v>b2fafe20fb3eb989ba21e613d6edab015456ffd2928eb6eaadbfbe2d16a1ce11</x:v>
-      </x:c>
-      <x:c r="G32" s="17" t="str">
-        <x:v>Superseded by: RFC-012</x:v>
-      </x:c>
-      <x:c r="H32" s="17" t="str">
+      <x:c r="F32" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G32" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H32" s="20" t="str">
+        <x:v>18b444d8e1c2c5b21c12c45a797973bea066283817ace847b549bd14f4b72578</x:v>
+      </x:c>
+      <x:c r="I32" s="17" t="str">
+        <x:v>Superseded by: ESM-001 v1.2</x:v>
+      </x:c>
+      <x:c r="J32" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="32" customHeight="1">
       <x:c r="A33" s="17" t="str">
-        <x:v>architecture/released/v1.0/SRM-001_Semantic_Resolution_Business_Capability_Specification_v1.0_FROZEN.docx</x:v>
+        <x:v>architecture/released/v1.0/GEM-001_Governance_Exception_Business_Specification_v1.0_FROZEN.docx</x:v>
       </x:c>
       <x:c r="B33" s="17" t="str">
-        <x:v>SRM-001</x:v>
+        <x:v>GEM-001</x:v>
       </x:c>
       <x:c r="C33" s="17" t="str">
-        <x:v>SRM-001 Semantic Resolution Business Capability Specification</x:v>
+        <x:v>GEM-001 Governance Exception Business Specification</x:v>
       </x:c>
       <x:c r="D33" s="19" t="str">
         <x:v>1.0</x:v>
@@ -1148,51 +1328,733 @@
       <x:c r="E33" s="18" t="str">
         <x:v>Superseded</x:v>
       </x:c>
-      <x:c r="F33" s="20" t="str">
-        <x:v>3e6cc26599fcdde3076e6d90bbf50a1e994416288bbeb38974d26c84abdde3fa</x:v>
-      </x:c>
-      <x:c r="G33" s="17" t="str">
-        <x:v>Superseded by: SRM-001 v2.0</x:v>
-      </x:c>
-      <x:c r="H33" s="17" t="str">
+      <x:c r="F33" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G33" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H33" s="20" t="str">
+        <x:v>84c45b69ef9afb01ee32775750b09f6e2e118a98a6effd2d329a87e66f70e35e</x:v>
+      </x:c>
+      <x:c r="I33" s="17" t="str">
+        <x:v>Superseded by: GEM-001 v1.1</x:v>
+      </x:c>
+      <x:c r="J33" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="32" customHeight="1">
       <x:c r="A34" s="17" t="str">
+        <x:v>architecture/released/v1.0/GRM-001_Governance_Business_Capability_Specification_v1.1_FROZEN.docx</x:v>
+      </x:c>
+      <x:c r="B34" s="17" t="str">
+        <x:v>GRM-001</x:v>
+      </x:c>
+      <x:c r="C34" s="17" t="str">
+        <x:v>GRM-001 Governance Business Capability Specification</x:v>
+      </x:c>
+      <x:c r="D34" s="19" t="str">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="E34" s="18" t="str">
+        <x:v>Superseded</x:v>
+      </x:c>
+      <x:c r="F34" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G34" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H34" s="20" t="str">
+        <x:v>da290fd2bb521b278f9a245a8111da9eeddd6fec817596bdc6c57d68d1bffff3</x:v>
+      </x:c>
+      <x:c r="I34" s="17" t="str">
+        <x:v>Superseded by: GRM-001 v1.2</x:v>
+      </x:c>
+      <x:c r="J34" s="17" t="str">
+        <x:v>Architecture Registry v1.0 release decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="32" customHeight="1">
+      <x:c r="A35" s="17" t="str">
+        <x:v>architecture/released/v1.0/KRM-001_Knowledge_Business_Capability_Specification_v1.2_FROZEN.docx</x:v>
+      </x:c>
+      <x:c r="B35" s="17" t="str">
+        <x:v>KRM-001</x:v>
+      </x:c>
+      <x:c r="C35" s="17" t="str">
+        <x:v>KRM-001 Knowledge Business Capability Specification</x:v>
+      </x:c>
+      <x:c r="D35" s="19" t="str">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="E35" s="18" t="str">
+        <x:v>Superseded</x:v>
+      </x:c>
+      <x:c r="F35" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G35" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H35" s="20" t="str">
+        <x:v>411299c35ef7affd06dfa250eadddd60d1e5edbe9568933cfeb0ac0c7b8adde2</x:v>
+      </x:c>
+      <x:c r="I35" s="17" t="str">
+        <x:v>Superseded by: KRM-001 v1.3</x:v>
+      </x:c>
+      <x:c r="J35" s="17" t="str">
+        <x:v>Architecture Registry v1.0 release decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="32" customHeight="1">
+      <x:c r="A36" s="17" t="str">
+        <x:v>architecture/released/v1.0/KRM-001_Knowledge_Business_Capability_Specification_v1.3_FROZEN.docx</x:v>
+      </x:c>
+      <x:c r="B36" s="17" t="str">
+        <x:v>KRM-001</x:v>
+      </x:c>
+      <x:c r="C36" s="17" t="str">
+        <x:v>KRM-001 Knowledge Business Capability Specification</x:v>
+      </x:c>
+      <x:c r="D36" s="19" t="str">
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="E36" s="18" t="str">
+        <x:v>Superseded</x:v>
+      </x:c>
+      <x:c r="F36" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G36" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H36" s="20" t="str">
+        <x:v>9b276dc8cf99e3aac3284717edc78991570f849589a748672b7da496b65fe832</x:v>
+      </x:c>
+      <x:c r="I36" s="17" t="str">
+        <x:v>Superseded by: KRM-001 v1.4</x:v>
+      </x:c>
+      <x:c r="J36" s="17" t="str">
+        <x:v>Architecture Registry v1.0 release decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="32" customHeight="1">
+      <x:c r="A37" s="17" t="str">
+        <x:v>architecture/released/v1.0/PAD-001_Product_Access_Architecture_v1.0_FROZEN.docx</x:v>
+      </x:c>
+      <x:c r="B37" s="17" t="str">
+        <x:v>PAD-001 Product Access Architecture</x:v>
+      </x:c>
+      <x:c r="C37" s="17" t="str">
+        <x:v>PAD-001 Product Access Architecture</x:v>
+      </x:c>
+      <x:c r="D37" s="19" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="E37" s="18" t="str">
+        <x:v>Superseded</x:v>
+      </x:c>
+      <x:c r="F37" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G37" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H37" s="20" t="str">
+        <x:v>705c30b0f4c8c755f3e6e46eba9c7974d0e827a664c573e23d05b13d9617a710</x:v>
+      </x:c>
+      <x:c r="I37" s="17" t="str">
+        <x:v>Superseded by: PAD-001 Protocol v1.1</x:v>
+      </x:c>
+      <x:c r="J37" s="17" t="str">
+        <x:v>Architecture Registry v1.0 release decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="32" customHeight="1">
+      <x:c r="A38" s="17" t="str">
+        <x:v>architecture/released/v1.0/PAD-001_Product_Access_Protocol_Specification_v1.1_FROZEN.docx</x:v>
+      </x:c>
+      <x:c r="B38" s="17" t="str">
+        <x:v>PAD-001 Product Access Protocol</x:v>
+      </x:c>
+      <x:c r="C38" s="17" t="str">
+        <x:v>PAD-001 Product Access Protocol Specification</x:v>
+      </x:c>
+      <x:c r="D38" s="19" t="str">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="E38" s="18" t="str">
+        <x:v>Superseded</x:v>
+      </x:c>
+      <x:c r="F38" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G38" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H38" s="20" t="str">
+        <x:v>a19c88bfeaddc8d391bb46338f6f7c179d30af6154772082ebca4835b2ce5948</x:v>
+      </x:c>
+      <x:c r="I38" s="17" t="str">
+        <x:v>Superseded by: PAD-001 v1.2</x:v>
+      </x:c>
+      <x:c r="J38" s="17" t="str">
+        <x:v>Architecture Registry v1.0 release decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="32" customHeight="1">
+      <x:c r="A39" s="17" t="str">
+        <x:v>architecture/released/v1.0/PAD-001_Product_Access_Protocol_Specification_v1.2_FROZEN.docx</x:v>
+      </x:c>
+      <x:c r="B39" s="17" t="str">
+        <x:v>PAD-001 Product Access Protocol</x:v>
+      </x:c>
+      <x:c r="C39" s="17" t="str">
+        <x:v>PAD-001 Product Access Protocol Specification</x:v>
+      </x:c>
+      <x:c r="D39" s="19" t="str">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="E39" s="18" t="str">
+        <x:v>Superseded</x:v>
+      </x:c>
+      <x:c r="F39" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G39" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H39" s="20" t="str">
+        <x:v>496ee104092949a5245aca0a0a4862f3a14f7b244d6e3792c9b70ecf53172f2a</x:v>
+      </x:c>
+      <x:c r="I39" s="17" t="str">
+        <x:v>Superseded by: PAD-001 v1.3</x:v>
+      </x:c>
+      <x:c r="J39" s="17" t="str">
+        <x:v>Architecture Registry v1.0 release decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="32" customHeight="1">
+      <x:c r="A40" s="17" t="str">
+        <x:v>architecture/released/v1.0/PAD-001_Product_Access_Protocol_Specification_v1.3_FROZEN.docx</x:v>
+      </x:c>
+      <x:c r="B40" s="17" t="str">
+        <x:v>PAD-001 Product Access Protocol</x:v>
+      </x:c>
+      <x:c r="C40" s="17" t="str">
+        <x:v>PAD-001 Product Access Protocol Specification</x:v>
+      </x:c>
+      <x:c r="D40" s="19" t="str">
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="E40" s="18" t="str">
+        <x:v>Superseded</x:v>
+      </x:c>
+      <x:c r="F40" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G40" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H40" s="20" t="str">
+        <x:v>2a11906e0c759c787f0a6dfc1c2cc9810e34a097aad4a8b4dca2c3f2e599ad06</x:v>
+      </x:c>
+      <x:c r="I40" s="17" t="str">
+        <x:v>Superseded by: PAD-001 v1.4</x:v>
+      </x:c>
+      <x:c r="J40" s="17" t="str">
+        <x:v>Architecture Registry v1.0 release decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="32" customHeight="1">
+      <x:c r="A41" s="17" t="str">
+        <x:v>architecture/released/v1.0/README.md</x:v>
+      </x:c>
+      <x:c r="B41" s="17" t="str">
+        <x:v>RELEASE-README</x:v>
+      </x:c>
+      <x:c r="C41" s="17" t="str">
+        <x:v>Architecture Release Baseline README</x:v>
+      </x:c>
+      <x:c r="D41" s="19" t="str">
+        <x:v>v1.0</x:v>
+      </x:c>
+      <x:c r="E41" s="18" t="str">
+        <x:v>Historical</x:v>
+      </x:c>
+      <x:c r="F41" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G41" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H41" s="20" t="str">
+        <x:v>62dbb300a104238c4ec86ee58ff631a7359b6dca18b99ed6fe981685e194fdb8</x:v>
+      </x:c>
+      <x:c r="I41" s="17" t="str"/>
+      <x:c r="J41" s="17" t="str">
+        <x:v>Architecture Registry v1.0 release decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="32" customHeight="1">
+      <x:c r="A42" s="17" t="str">
+        <x:v>architecture/released/v1.0/RELEASE-READINESS-REPORT-v1.1_FROZEN.md</x:v>
+      </x:c>
+      <x:c r="B42" s="17" t="str">
+        <x:v>Release Readiness Report</x:v>
+      </x:c>
+      <x:c r="C42" s="17" t="str">
+        <x:v>RELEASE-READINESS-REPORT-v1.1</x:v>
+      </x:c>
+      <x:c r="D42" s="19" t="str">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="E42" s="18" t="str">
+        <x:v>Superseded</x:v>
+      </x:c>
+      <x:c r="F42" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G42" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H42" s="20" t="str">
+        <x:v>1bc78e656b64f5292090cd491cd4541ce550f5d621ae3f0aa60f961440940977</x:v>
+      </x:c>
+      <x:c r="I42" s="17" t="str">
+        <x:v>Superseded by: RRR-001 v1.2</x:v>
+      </x:c>
+      <x:c r="J42" s="17" t="str">
+        <x:v>Architecture Registry v1.0 release decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="32" customHeight="1">
+      <x:c r="A43" s="17" t="str">
+        <x:v>architecture/released/v1.0/RFC-0001 - Enterprise Knowledge Specification v1.0.docx</x:v>
+      </x:c>
+      <x:c r="B43" s="17" t="str">
+        <x:v>RFC-0001</x:v>
+      </x:c>
+      <x:c r="C43" s="17" t="str">
+        <x:v>RFC-0001 - Enterprise Knowledge Specification</x:v>
+      </x:c>
+      <x:c r="D43" s="19" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="E43" s="18" t="str">
+        <x:v>Superseded</x:v>
+      </x:c>
+      <x:c r="F43" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G43" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H43" s="20" t="str">
+        <x:v>05be0b62e53744708d5268080406ec2e78c6ff5e541e657b3e11e3a98f18580c</x:v>
+      </x:c>
+      <x:c r="I43" s="17" t="str">
+        <x:v>Superseded by: RFC-012</x:v>
+      </x:c>
+      <x:c r="J43" s="17" t="str">
+        <x:v>Architecture Registry v1.0 release decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="32" customHeight="1">
+      <x:c r="A44" s="17" t="str">
+        <x:v>architecture/released/v1.0/RFC-0002 - Enterprise Ontology Specification v1.0.docx</x:v>
+      </x:c>
+      <x:c r="B44" s="17" t="str">
+        <x:v>RFC-0002</x:v>
+      </x:c>
+      <x:c r="C44" s="17" t="str">
+        <x:v>RFC-0002 - Enterprise Ontology Specification</x:v>
+      </x:c>
+      <x:c r="D44" s="19" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="E44" s="18" t="str">
+        <x:v>Superseded</x:v>
+      </x:c>
+      <x:c r="F44" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G44" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H44" s="20" t="str">
+        <x:v>37c4efb92df9a5fd40d9b140971d6e482a06d712a6747ab455f3bc86b0e3aaff</x:v>
+      </x:c>
+      <x:c r="I44" s="17" t="str">
+        <x:v>Superseded by: RFC-012</x:v>
+      </x:c>
+      <x:c r="J44" s="17" t="str">
+        <x:v>Architecture Registry v1.0 release decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="32" customHeight="1">
+      <x:c r="A45" s="17" t="str">
+        <x:v>architecture/released/v1.0/RFC-0003 - Institutional Acts Specification v1.0.docx</x:v>
+      </x:c>
+      <x:c r="B45" s="17" t="str">
+        <x:v>RFC-0003</x:v>
+      </x:c>
+      <x:c r="C45" s="17" t="str">
+        <x:v>RFC-0003 - Institutional Acts Specification</x:v>
+      </x:c>
+      <x:c r="D45" s="19" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="E45" s="18" t="str">
+        <x:v>Superseded</x:v>
+      </x:c>
+      <x:c r="F45" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G45" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H45" s="20" t="str">
+        <x:v>2d130363c663e80c4ee4be3ad01961a69eed619d24bd5688f2cfa59017c72279</x:v>
+      </x:c>
+      <x:c r="I45" s="17" t="str">
+        <x:v>Superseded by: RFC-012</x:v>
+      </x:c>
+      <x:c r="J45" s="17" t="str">
+        <x:v>Architecture Registry v1.0 release decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="32" customHeight="1">
+      <x:c r="A46" s="17" t="str">
+        <x:v>architecture/released/v1.0/RFC-0004 - Enterprise Knowledge Graph Specification v1.0.docx</x:v>
+      </x:c>
+      <x:c r="B46" s="17" t="str">
+        <x:v>RFC-0004</x:v>
+      </x:c>
+      <x:c r="C46" s="17" t="str">
+        <x:v>RFC-0004 - Enterprise Knowledge Graph Specification</x:v>
+      </x:c>
+      <x:c r="D46" s="19" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="E46" s="18" t="str">
+        <x:v>Superseded</x:v>
+      </x:c>
+      <x:c r="F46" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G46" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H46" s="20" t="str">
+        <x:v>0f8162d2dceb1e1b544bb7bb2cd0eae11c6c07f84e2f3b81c30f6699927f0874</x:v>
+      </x:c>
+      <x:c r="I46" s="17" t="str">
+        <x:v>Superseded by: RFC-012</x:v>
+      </x:c>
+      <x:c r="J46" s="17" t="str">
+        <x:v>Architecture Registry v1.0 release decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="32" customHeight="1">
+      <x:c r="A47" s="17" t="str">
+        <x:v>architecture/released/v1.0/RFC-0005 - Decision Assembly Specification v1.0.docx</x:v>
+      </x:c>
+      <x:c r="B47" s="17" t="str">
+        <x:v>RFC-0005</x:v>
+      </x:c>
+      <x:c r="C47" s="17" t="str">
+        <x:v>RFC-0005 - Decision Assembly Specification</x:v>
+      </x:c>
+      <x:c r="D47" s="19" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="E47" s="18" t="str">
+        <x:v>Superseded</x:v>
+      </x:c>
+      <x:c r="F47" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G47" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H47" s="20" t="str">
+        <x:v>756eb0ee4d57cbd5795ca56f31ba3b479431eaf3e31abfd480e5d21765bbc8a5</x:v>
+      </x:c>
+      <x:c r="I47" s="17" t="str">
+        <x:v>Superseded by: RFC-012</x:v>
+      </x:c>
+      <x:c r="J47" s="17" t="str">
+        <x:v>Architecture Registry v1.0 release decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="32" customHeight="1">
+      <x:c r="A48" s="17" t="str">
+        <x:v>architecture/released/v1.0/RFC-0006 - Enterprise Memory Specification v1.0.docx</x:v>
+      </x:c>
+      <x:c r="B48" s="17" t="str">
+        <x:v>RFC-0006</x:v>
+      </x:c>
+      <x:c r="C48" s="17" t="str">
+        <x:v>RFC-0006 - Enterprise Memory Specification</x:v>
+      </x:c>
+      <x:c r="D48" s="19" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="E48" s="18" t="str">
+        <x:v>Superseded</x:v>
+      </x:c>
+      <x:c r="F48" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G48" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H48" s="20" t="str">
+        <x:v>853578f062a3f8d6662f50d6fa8535ce5c0c5e992ee14a7599432cfa3b6b6933</x:v>
+      </x:c>
+      <x:c r="I48" s="17" t="str">
+        <x:v>Superseded by: RFC-012</x:v>
+      </x:c>
+      <x:c r="J48" s="17" t="str">
+        <x:v>Architecture Registry v1.0 release decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="32" customHeight="1">
+      <x:c r="A49" s="17" t="str">
+        <x:v>architecture/released/v1.0/RFC-0007 - Enterprise Reasoning Specification v1.0.docx</x:v>
+      </x:c>
+      <x:c r="B49" s="17" t="str">
+        <x:v>RFC-0007</x:v>
+      </x:c>
+      <x:c r="C49" s="17" t="str">
+        <x:v>RFC-0007 - Enterprise Reasoning Specification</x:v>
+      </x:c>
+      <x:c r="D49" s="19" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="E49" s="18" t="str">
+        <x:v>Superseded</x:v>
+      </x:c>
+      <x:c r="F49" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G49" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H49" s="20" t="str">
+        <x:v>370b47e8fbfba8ec34afaf78e7cb4c11cd6b5ca19e8605f21a8649491e1712ed</x:v>
+      </x:c>
+      <x:c r="I49" s="17" t="str">
+        <x:v>Superseded by: RFC-012</x:v>
+      </x:c>
+      <x:c r="J49" s="17" t="str">
+        <x:v>Architecture Registry v1.0 release decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="32" customHeight="1">
+      <x:c r="A50" s="17" t="str">
+        <x:v>architecture/released/v1.0/RFC-0008 - Enterprise Decision Specification v1.0.docx</x:v>
+      </x:c>
+      <x:c r="B50" s="17" t="str">
+        <x:v>RFC-0008</x:v>
+      </x:c>
+      <x:c r="C50" s="17" t="str">
+        <x:v>RFC-0008 - Enterprise Decision Specification</x:v>
+      </x:c>
+      <x:c r="D50" s="19" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="E50" s="18" t="str">
+        <x:v>Superseded</x:v>
+      </x:c>
+      <x:c r="F50" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G50" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H50" s="20" t="str">
+        <x:v>88850719c91374469a930ac5420232e45df78c821ad5515cb00dd7c6ebc45fcb</x:v>
+      </x:c>
+      <x:c r="I50" s="17" t="str">
+        <x:v>Superseded by: RFC-012</x:v>
+      </x:c>
+      <x:c r="J50" s="17" t="str">
+        <x:v>Architecture Registry v1.0 release decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="32" customHeight="1">
+      <x:c r="A51" s="17" t="str">
+        <x:v>architecture/released/v1.0/RFC-0009 - Enterprise Learning Specification v1.0.docx</x:v>
+      </x:c>
+      <x:c r="B51" s="17" t="str">
+        <x:v>RFC-0009</x:v>
+      </x:c>
+      <x:c r="C51" s="17" t="str">
+        <x:v>RFC-0009 - Enterprise Learning Specification</x:v>
+      </x:c>
+      <x:c r="D51" s="19" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="E51" s="18" t="str">
+        <x:v>Superseded</x:v>
+      </x:c>
+      <x:c r="F51" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G51" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H51" s="20" t="str">
+        <x:v>b2fafe20fb3eb989ba21e613d6edab015456ffd2928eb6eaadbfbe2d16a1ce11</x:v>
+      </x:c>
+      <x:c r="I51" s="17" t="str">
+        <x:v>Superseded by: RFC-012</x:v>
+      </x:c>
+      <x:c r="J51" s="17" t="str">
+        <x:v>Architecture Registry v1.0 release decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="32" customHeight="1">
+      <x:c r="A52" s="17" t="str">
+        <x:v>architecture/released/v1.0/RFC-013_Governance_Authority_and_Evaluation_Separation_v1.0_FROZEN.docx</x:v>
+      </x:c>
+      <x:c r="B52" s="17" t="str">
+        <x:v>RFC-013</x:v>
+      </x:c>
+      <x:c r="C52" s="17" t="str">
+        <x:v>RFC-013 Governance Authority and Evaluation Separation</x:v>
+      </x:c>
+      <x:c r="D52" s="19" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="E52" s="18" t="str">
+        <x:v>Superseded</x:v>
+      </x:c>
+      <x:c r="F52" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G52" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H52" s="20" t="str">
+        <x:v>3ea499c07d4998c542ccd5c17b02b0163f570e15d0fb3faf6fc03df31dd1b9c1</x:v>
+      </x:c>
+      <x:c r="I52" s="17" t="str">
+        <x:v>Superseded by: RFC-013 v1.1</x:v>
+      </x:c>
+      <x:c r="J52" s="17" t="str">
+        <x:v>Architecture Registry v1.0 release decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="32" customHeight="1">
+      <x:c r="A53" s="17" t="str">
+        <x:v>architecture/released/v1.0/SRM-001_Semantic_Resolution_Business_Capability_Specification_v1.0_FROZEN.docx</x:v>
+      </x:c>
+      <x:c r="B53" s="17" t="str">
+        <x:v>SRM-001</x:v>
+      </x:c>
+      <x:c r="C53" s="17" t="str">
+        <x:v>SRM-001 Semantic Resolution Business Capability Specification</x:v>
+      </x:c>
+      <x:c r="D53" s="19" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="E53" s="18" t="str">
+        <x:v>Superseded</x:v>
+      </x:c>
+      <x:c r="F53" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G53" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H53" s="20" t="str">
+        <x:v>3e6cc26599fcdde3076e6d90bbf50a1e994416288bbeb38974d26c84abdde3fa</x:v>
+      </x:c>
+      <x:c r="I53" s="17" t="str">
+        <x:v>Superseded by: SRM-001 v2.0</x:v>
+      </x:c>
+      <x:c r="J53" s="17" t="str">
+        <x:v>Architecture Registry v1.0 release decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="32" customHeight="1">
+      <x:c r="A54" s="17" t="str">
         <x:v>architecture/released/v1.0/SRM-001_Semantic_Resolution_Business_Capability_Specification_v2.0_FROZEN.docx</x:v>
       </x:c>
-      <x:c r="B34" s="17" t="str">
+      <x:c r="B54" s="17" t="str">
         <x:v>SRM-001</x:v>
       </x:c>
-      <x:c r="C34" s="17" t="str">
+      <x:c r="C54" s="17" t="str">
         <x:v>SRM-001 Semantic Resolution Business Capability Specification</x:v>
       </x:c>
-      <x:c r="D34" s="19" t="str">
+      <x:c r="D54" s="19" t="str">
         <x:v>2.0</x:v>
       </x:c>
-      <x:c r="E34" s="18" t="str">
-        <x:v>Superseded</x:v>
-      </x:c>
-      <x:c r="F34" s="20" t="str">
+      <x:c r="E54" s="18" t="str">
+        <x:v>Superseded</x:v>
+      </x:c>
+      <x:c r="F54" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G54" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H54" s="20" t="str">
         <x:v>ced6e640823ba1896368d9f0ba0c3c719d0a85bfcf93dc115f08a032ea1463f6</x:v>
       </x:c>
-      <x:c r="G34" s="17" t="str">
+      <x:c r="I54" s="17" t="str">
         <x:v>Superseded by: SRM-001 v2.1</x:v>
       </x:c>
-      <x:c r="H34" s="17" t="str">
+      <x:c r="J54" s="17" t="str">
+        <x:v>Architecture Registry v1.0 release decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="32" customHeight="1">
+      <x:c r="A55" s="17" t="str">
+        <x:v>architecture/released/v1.0/SRM-001_Semantic_Resolution_Business_Capability_Specification_v2.1_FROZEN.docx</x:v>
+      </x:c>
+      <x:c r="B55" s="17" t="str">
+        <x:v>SRM-001</x:v>
+      </x:c>
+      <x:c r="C55" s="17" t="str">
+        <x:v>SRM-001 Semantic Resolution Business Capability Specification</x:v>
+      </x:c>
+      <x:c r="D55" s="19" t="str">
+        <x:v>2.1</x:v>
+      </x:c>
+      <x:c r="E55" s="18" t="str">
+        <x:v>Superseded</x:v>
+      </x:c>
+      <x:c r="F55" s="18" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G55" s="18" t="str">
+        <x:v>NON-AUTHORITATIVE</x:v>
+      </x:c>
+      <x:c r="H55" s="20" t="str">
+        <x:v>004e3861626a8bcace8524c7f2aa1573938ec9840bacd45088efaa38c8fa0eb7</x:v>
+      </x:c>
+      <x:c r="I55" s="17" t="str">
+        <x:v>Superseded by: SRM-001 v2.2</x:v>
+      </x:c>
+      <x:c r="J55" s="17" t="str">
         <x:v>Architecture Registry v1.0 release decision</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
-    <x:mergeCell ref="E3:H3"/>
+    <x:mergeCell ref="A1:J1"/>
+    <x:mergeCell ref="A2:J2"/>
+    <x:mergeCell ref="E3:J3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b2b21ff2ae242d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re57fa738f8f64074"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>